<commit_message>
Modify Zicsr TP to add assertible case
</commit_message>
<xml_diff>
--- a/coretp/plans/zicsr/Zicsr_TP.xlsx
+++ b/coretp/plans/zicsr/Zicsr_TP.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njoaquin/Documents/Clean Test Plans/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njoaquin/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{828B6BA9-94B1-C745-BE3D-78E931206DE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77C42DDA-38FC-9341-B228-9F5118A30F3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34560" yWindow="-14220" windowWidth="51200" windowHeight="28800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="40" yWindow="760" windowWidth="34560" windowHeight="20540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Zicsr" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="76">
   <si>
     <t>Scenario details</t>
   </si>
@@ -357,12 +357,62 @@
 CsrDirectAccess(op="csrrci", csr_name=None, src1=None, target_is_x0=False)
 CsrDirectAccess(op="csrrci", csr_name=None, src1=None, target_is_x0=False)</t>
   </si>
+  <si>
+    <t>SID_ZICSR_18</t>
+  </si>
+  <si>
+    <t>Assert Case</t>
+  </si>
+  <si>
+    <t>Using Scratch registers, test CSRRW{I}/CSRRS{I}/CSRRC{I}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Comment(comment="ZICSR test: mscratch write/set/clear with assertions (M-mode)")                                                                                                                   
+  LoadImmediateStep(imm=-1)
+  LoadImmediateStep(imm=0)                                                                                                                                                                           
+  LoadImmediateStep(imm=0x1F)
+  Comment(comment="CSRRW: Write all ones to mscratch")
+  CsrDirectAccess(op="csrrw", csr_name="mscratch", src1=all_ones, target_is_x0=False)
+  CsrRead(csr_name="mscratch", direct_read=True)
+  AssertEqual(src1=read_after_csrrw, src2=all_ones)
+  Comment(comment="CSRRW: Clear mscratch by writing 0")
+  CsrDirectAccess(op="csrrw", csr_name="mscratch", src1=0, target_is_x0=False)
+  CsrRead(csr_name="mscratch", direct_read=True)
+  AssertEqual(src1=read_after_csrrw_clear, src2=zero)
+  Comment(comment="CSRRS: Set all bits in mscratch")
+  CsrDirectAccess(op="csrrs", csr_name="mscratch", src1=all_ones, target_is_x0=False)
+  CsrRead(csr_name="mscratch", direct_read=True)
+  AssertEqual(src1=read_after_csrrs, src2=all_ones)
+  Comment(comment="CSRRC: Clear all bits in mscratch")
+  CsrDirectAccess(op="csrrc", csr_name="mscratch", src1=all_ones, target_is_x0=False)
+  CsrRead(csr_name="mscratch", direct_read=True)
+  AssertEqual(src1=read_after_csrrc, src2=zero)
+  Comment(comment="CSRRWI: Write max immediate (0x1F) to mscratch")
+  CsrDirectAccess(op="csrrwi", csr_name="mscratch", src1=0x1F, target_is_x0=False)
+  CsrRead(csr_name="mscratch", direct_read=True)
+  AssertEqual(src1=read_after_csrrwi, src2=max_imm)
+  Comment(comment="CSRRWI: Clear mscratch by writing 0")
+  CsrDirectAccess(op="csrrwi", csr_name="mscratch", src1=0, target_is_x0=False)
+  CsrRead(csr_name="mscratch", direct_read=True)
+  AssertEqual(src1=read_after_csrrwi_clear, src2=zero)
+  Comment(comment="CSRRSI: Set bits with max immediate (0x1F) in mscratch")
+  CsrDirectAccess(op="csrrsi", csr_name="mscratch", src1=0x1F, target_is_x0=False)
+  CsrRead(csr_name="mscratch", direct_read=True)
+  AssertEqual(src1=read_after_csrrsi, src2=max_imm)
+  Comment(comment="CSRRCI: Clear bits with max immediate (0x1F) in mscratch")
+  CsrDirectAccess(op="csrrci", csr_name="mscratch", src1=0x1F, target_is_x0=False)
+  CsrRead(csr_name="mscratch", direct_read=True)
+  AssertEqual(src1=read_after_csrrci, src2=zero)</t>
+  </si>
+  <si>
+    <t>mscratch/sscratch/fcsr (for each mode)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -403,6 +453,11 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri (Body)"/>
     </font>
   </fonts>
   <fills count="5">
@@ -515,7 +570,7 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -528,6 +583,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="2" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -851,7 +909,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62A8FE57-9C2B-4CE6-9C64-CA961B39B2D9}">
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.6640625" bestFit="1" customWidth="1"/>
@@ -863,13 +921,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
       <c r="F1" s="5"/>
     </row>
     <row r="2" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -1159,7 +1217,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" ht="409.5" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
         <v>52</v>
       </c>
@@ -1174,6 +1232,23 @@
       </c>
       <c r="E19" s="1" t="s">
         <v>70</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A20" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B20" t="s">
+        <v>72</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>